<commit_message>
Update bulk import template
Changed Phonenumber Restrictions:
-no letters
-fixed length
</commit_message>
<xml_diff>
--- a/public/templates/bulk-import-template.xlsx
+++ b/public/templates/bulk-import-template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_4E22B6AF77BEABA23143F343374451B34654107B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{016A3140-8D4B-41F7-9729-21A6DFC94B44}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_D69F3177706D7D87E743F36727ECBC2F22D0338F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{407AB83F-9BDA-4E13-868F-72C5E942061A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>firstName</t>
   </si>
@@ -41,7 +41,7 @@
     <t>jane.smith@example.com</t>
   </si>
   <si>
-    <t>0400000000</t>
+    <t>Student</t>
   </si>
   <si>
     <t>Mary-Jane</t>
@@ -53,13 +53,10 @@
     <t>mary-jane.doe@example.com</t>
   </si>
   <si>
-    <t>0400000001</t>
-  </si>
-  <si>
-    <t>Student</t>
-  </si>
-  <si>
     <t>Tutor</t>
+  </si>
+  <si>
+    <t>0412345678</t>
   </si>
 </sst>
 </file>
@@ -100,9 +97,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -118,6 +117,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -442,33 +445,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -478,14 +481,14 @@
       <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -495,20 +498,43 @@
       <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
     </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25"/>
+    <row r="17" x14ac:dyDescent="0.25"/>
+    <row r="18" x14ac:dyDescent="0.25"/>
+    <row r="19" x14ac:dyDescent="0.25"/>
+    <row r="20" x14ac:dyDescent="0.25"/>
+    <row r="21" x14ac:dyDescent="0.25"/>
+    <row r="22" x14ac:dyDescent="0.25"/>
+    <row r="23" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid role" error="Role must be one of: client, student, tutor, coordinator, liaison" sqref="E2:E1051" xr:uid="{B0264E20-8DB1-48DD-960B-B3CCC4C4CD39}">
+  <dataValidations count="2">
+    <dataValidation type="custom" allowBlank="1" showErrorMessage="1" errorTitle="Invalid phone number" error="Phone number must be in the format 0400000000 (starts with 0, 10 digits total)." sqref="D2:D201" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>AND(LEN(D2)=10,LEFT(D2,1)="0",ISNUMBER(VALUE(MID(D2,2,9))))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid role" error="Role must be one of: client, student, tutor, coordinator, liaison" sqref="E2:E1051" xr:uid="{00000000-0002-0000-0000-0000C8000000}">
       <formula1>"Client,Student,Tutor,Unit Coordinator,Liaison"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>